<commit_message>
📊 Horarios actualizados Línea 141 - 1332
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:22:54</t>
+          <t>Última actualización: 12:42:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>13:01</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>13:01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,12 +723,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -753,16 +753,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13:46</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>84</v>
+        <v>39</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>114</v>
+        <v>63</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -978,18 +978,243 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>13:46</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>84</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>65</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>69</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>77</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>14:16</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D30" t="n">
+        <v>94</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>12:22:54</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
         <v>114</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>95</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>96</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>110</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>116</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1006,7 +1231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1019,14 +1244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:22:54</t>
+          <t>Última actualización: 12:42:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1310,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1099,7 +1324,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1110,7 +1335,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1124,7 +1349,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1135,7 +1360,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1149,9 +1374,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>96</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1181,7 +1431,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:22:54</t>
+          <t>Última actualización: 12:42:43</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1472,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1236,7 +1486,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1247,7 +1497,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1261,7 +1511,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1272,7 +1522,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1286,7 +1536,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1297,7 +1547,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1311,7 +1561,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1333
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:43</t>
+          <t>Última actualización: 12:56:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>13:06</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -828,16 +828,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:22:54</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -928,16 +928,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:19</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>13:46</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>84</v>
+        <v>25</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1053,16 +1053,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:22:54</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:46</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,23 +1198,273 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>63</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>12:42:43</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>94</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>12:22:54</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>114</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>81</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>81</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>96</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>83</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>110</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>97</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>14:38</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>116</v>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D44" t="n">
+        <v>102</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>115</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1231,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1244,14 +1494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:43</t>
+          <t>Última actualización: 12:56:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1335,21 +1585,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1365,16 +1615,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1385,23 +1635,123 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>23</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>12:42:43</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>42</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>14:18</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D13" t="n">
         <v>96</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>83</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1418,7 +1768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1431,14 +1781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:43</t>
+          <t>Última actualización: 12:56:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1497,25 +1847,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -1527,16 +1877,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1547,23 +1897,123 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>12:42:43</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>39</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>26</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>13:55</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D12" t="n">
         <v>73</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>60</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1334
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:56:14</t>
+          <t>Última actualización: 13:17:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,12 +948,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -978,16 +978,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:19</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,12 +1023,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>13:46</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1178,16 +1178,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:22:54</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:46</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>63</v>
+        <v>84</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>94</v>
+        <v>30</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>96</v>
+        <v>46</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:22:54</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>110</v>
+        <v>59</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,23 +1448,223 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>61</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>12:56:14</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>83</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>75</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>12:56:14</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>97</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>81</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>14:51</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>115</v>
-      </c>
-      <c r="E45" t="inlineStr">
+      <c r="D50" t="n">
+        <v>94</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>102</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>102</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>102</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1481,7 +1681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1494,14 +1694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:56:14</t>
+          <t>Última actualización: 13:17:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1810,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1624,7 +1824,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1660,7 +1860,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1674,7 +1874,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1710,7 +1910,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1724,7 +1924,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1752,6 +1952,31 @@
         <v>83</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>102</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1768,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1781,14 +2006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:56:14</t>
+          <t>Última actualización: 13:17:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -1922,7 +2147,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1936,7 +2161,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2016,6 +2241,81 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>43</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>88</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>108</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1335
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:17:49</t>
+          <t>Última actualización: 13:45:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>13:46</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,12 +1223,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>12:22:54</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:46</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>14:02</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1328,16 +1328,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>114</v>
+        <v>46</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:22:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1428,16 +1428,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:19</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>102</v>
+        <v>53</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,23 +1648,223 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>62</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>63</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>66</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>13:17:49</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>14:59</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>102</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>74</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>102</v>
-      </c>
-      <c r="E53" t="inlineStr">
+      <c r="D58" t="n">
+        <v>74</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>94</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>98</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>113</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1681,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1694,14 +1894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:17:49</t>
+          <t>Última actualización: 13:45:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -1935,7 +2135,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1949,7 +2149,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1960,7 +2160,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1974,9 +2174,34 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>94</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1993,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2006,14 +2231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:17:49</t>
+          <t>Última actualización: 13:45:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2247,12 +2472,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:57</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2261,7 +2486,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2277,7 +2502,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2286,7 +2511,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>88</v>
+        <v>43</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2302,18 +2527,93 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>88</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>61</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>15:05</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D18" t="n">
         <v>108</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>81</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1336
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:23</t>
+          <t>Última actualización: 13:58:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 67</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1298,12 +1298,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:58</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>14:02</t>
+          <t>13:58</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>12:22:54</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>114</v>
+        <v>46</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:06</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,12 +1473,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1553,16 +1553,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>14:21</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:19</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>63</v>
+        <v>97</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:37</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>102</v>
+        <v>53</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,18 +1853,293 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>66</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>60</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>13:17:49</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>102</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>74</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>61</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>80</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>13:45:23</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>94</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>85</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>15:38</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>113</v>
-      </c>
-      <c r="E61" t="inlineStr">
+      <c r="D69" t="n">
+        <v>100</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>15:50</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>112</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>115</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>118</v>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1881,7 +2156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1894,14 +2169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:23</t>
+          <t>Última actualización: 13:58:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2385,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2124,7 +2399,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2160,7 +2435,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2174,7 +2449,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2185,23 +2460,48 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>80</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>13:45:23</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>15:19</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>94</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2218,7 +2518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2231,14 +2531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:23</t>
+          <t>Última actualización: 13:58:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2822,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2536,7 +2836,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2572,7 +2872,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2586,7 +2886,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>108</v>
+        <v>67</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2616,6 +2916,31 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>107</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1337
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:57</t>
+          <t>Última actualización: 14:20:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 67</t>
+          <t>Total filas: 79</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>14:21</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>97</v>
+        <v>1</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>14:37</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:37</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1828,16 +1828,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>31</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>112</v>
+        <v>51</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2103,16 +2103,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,23 +2123,323 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>59</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>13:58:57</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>85</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>64</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>78</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>78</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>15:50</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>112</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>91</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>115</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>94</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
         <is>
           <t>15:56</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D72" t="n">
+      <c r="D81" t="n">
         <v>118</v>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>97</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>109</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>112</v>
+      </c>
+      <c r="E84" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2156,7 +2456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2169,14 +2469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:57</t>
+          <t>Última actualización: 14:20:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2435,21 +2735,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2465,16 +2765,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2485,23 +2785,73 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>80</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>15:19</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>94</v>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D19" t="n">
+        <v>59</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2518,7 +2868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2531,14 +2881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:57</t>
+          <t>Última actualización: 14:20:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2847,7 +3197,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2861,7 +3211,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2897,7 +3247,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2911,7 +3261,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2939,6 +3289,31 @@
         <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>86</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1338
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:20:09</t>
+          <t>Última actualización: 14:41:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 79</t>
+          <t>Total filas: 89</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,12 +1848,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1903,16 +1903,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,12 +1923,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>39</v>
+        <v>102</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,12 +2048,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2153,16 +2153,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2228,16 +2228,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>115</v>
+        <v>78</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>94</v>
+        <v>58</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>118</v>
+        <v>59</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>97</v>
+        <v>60</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>109</v>
+        <v>66</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,23 +2423,273 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
         <v>112</v>
       </c>
       <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>70</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>115</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>73</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>74</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>118</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>14:20:09</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>97</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>88</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>91</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>103</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>114</v>
+      </c>
+      <c r="E94" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2456,7 +2706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2469,14 +2719,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:20:09</t>
+          <t>Última actualización: 14:41:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2785,7 +3035,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2799,7 +3049,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2835,7 +3085,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2849,9 +3099,34 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>103</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2868,7 +3143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2881,14 +3156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:20:09</t>
+          <t>Última actualización: 14:41:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3472,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3211,7 +3486,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3272,48 +3547,73 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>35</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>107</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>14:41:17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>15:46</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>86</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D22" t="n">
+        <v>65</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1339
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:41:17</t>
+          <t>Última actualización: 14:55:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 89</t>
+          <t>Total filas: 96</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>64</v>
+        <v>24</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,12 +2298,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:33</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2312,7 +2312,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>15:39</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>115</v>
+        <v>52</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>73</v>
+        <v>112</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,23 +2673,198 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>15:59</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>64</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>74</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>76</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
           <t>14:41:17</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>91</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>89</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
         <is>
           <t>16:35</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D94" t="n">
-        <v>114</v>
-      </c>
-      <c r="E94" t="inlineStr">
+      <c r="D99" t="n">
+        <v>100</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>112</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>116</v>
+      </c>
+      <c r="E101" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2706,7 +2881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2719,14 +2894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:41:17</t>
+          <t>Última actualización: 14:55:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3010,12 +3185,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3024,7 +3199,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>61</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3035,12 +3210,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3049,7 +3224,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3060,21 +3235,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>80</v>
+        <v>19</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3085,12 +3260,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3099,7 +3274,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>38</v>
+        <v>80</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3110,23 +3285,48 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>24</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>16:24</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>103</v>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="D21" t="n">
+        <v>89</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3143,7 +3343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3156,14 +3356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:41:17</t>
+          <t>Última actualización: 14:55:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3572,50 +3772,125 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:17</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>107</v>
+        <v>22</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>13:58:57</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>107</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>14:41:17</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>15:46</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D23" t="n">
         <v>65</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>52</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>108</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1340
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:55:32</t>
+          <t>Última actualización: 15:18:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 96</t>
+          <t>Total filas: 103</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,12 +2273,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>15:33</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:33</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>78</v>
+        <v>17</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>43</v>
+        <v>78</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>15:39</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2428,16 +2428,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>112</v>
+        <v>29</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,12 +2523,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>56</v>
+        <v>112</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>115</v>
+        <v>33</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,12 +2623,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,12 +2648,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>97</v>
+        <v>38</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>64</v>
+        <v>97</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,12 +2748,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2762,7 +2762,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>91</v>
+        <v>53</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:12</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>112</v>
+        <v>65</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2853,18 +2853,193 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>89</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>77</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>79</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>89</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
           <t>16:51</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D101" t="n">
-        <v>116</v>
-      </c>
-      <c r="E101" t="inlineStr">
+      <c r="D105" t="n">
+        <v>93</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>101</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>101</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>17:11</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>113</v>
+      </c>
+      <c r="E108" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2881,7 +3056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2894,14 +3069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:55:32</t>
+          <t>Última actualización: 15:18:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3435,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3274,7 +3449,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3310,23 +3485,73 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>65</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>14:55:32</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>16:24</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D22" t="n">
         <v>89</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>101</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3343,7 +3568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3356,14 +3581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:55:32</t>
+          <t>Última actualización: 15:18:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -3797,37 +4022,37 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>107</v>
+        <v>3</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3836,7 +4061,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>65</v>
+        <v>107</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3847,12 +4072,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:46</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3861,7 +4086,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3877,20 +4102,120 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>52</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>30</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>84</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:55:32</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>16:43</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D28" t="n">
         <v>108</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>97</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1341
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:18:44</t>
+          <t>Última actualización: 15:51:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 103</t>
+          <t>Total filas: 118</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2548,7 +2548,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>74</v>
+        <v>3</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,12 +2648,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,12 +2673,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>97</v>
+        <v>5</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>41</v>
+        <v>97</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2728,16 +2728,16 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>14:41:17</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>91</v>
+        <v>13</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,16 +2803,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>14:41:17</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:12</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:13</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>16:37</t>
+          <t>16:22</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2928,16 +2928,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>93</v>
+        <v>32</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>101</v>
+        <v>44</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,23 +3023,398 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>44</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
           <t>15:18:44</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>79</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>47</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>55</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>89</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>60</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>68</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>68</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
         <is>
           <t>17:11</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D108" t="n">
-        <v>113</v>
-      </c>
-      <c r="E108" t="inlineStr">
+      <c r="D116" t="n">
+        <v>80</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>90</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>92</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>104</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>104</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>105</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>116</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>116</v>
+      </c>
+      <c r="E123" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3056,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3069,14 +3444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:18:44</t>
+          <t>Última actualización: 15:51:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3860,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3499,7 +3874,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3535,7 +3910,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3549,9 +3924,59 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>116</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>116</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3581,7 +4006,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:18:44</t>
+          <t>Última actualización: 15:51:56</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4572,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4161,7 +4586,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4197,7 +4622,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4211,7 +4636,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>97</v>
+        <v>64</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1342
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E123"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:51:56</t>
+          <t>Última actualización: 16:13:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 118</t>
+          <t>Total filas: 130</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>16:37</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,12 +3073,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,12 +3123,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>89</v>
+        <v>55</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>104</v>
+        <v>50</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3328,16 +3328,16 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>105</v>
+        <v>59</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>116</v>
+        <v>68</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,23 +3398,323 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>70</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>82</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>82</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>82</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
           <t>15:51:56</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>105</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>84</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>88</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>15:51:56</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
         <is>
           <t>17:47</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>116</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D123" t="n">
-        <v>116</v>
-      </c>
-      <c r="E123" t="inlineStr">
+      <c r="D131" t="n">
+        <v>94</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>95</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>98</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>106</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>107</v>
+      </c>
+      <c r="E135" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3431,7 +3731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3444,14 +3744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:51:56</t>
+          <t>Última actualización: 16:13:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3885,7 +4185,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3899,7 +4199,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3935,21 +4235,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>116</v>
+        <v>47</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3970,13 +4270,63 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>116</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>94</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>95</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3993,7 +4343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4006,14 +4356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:51:56</t>
+          <t>Última actualización: 16:13:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4947,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4611,7 +4961,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4639,6 +4989,31 @@
         <v>64</v>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>16:13:31</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>43</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1343
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E135"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:13:31</t>
+          <t>Última actualización: 16:34:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 130</t>
+          <t>Total filas: 134</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,12 +3073,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>16:37</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>79</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,12 +3098,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3112,7 +3112,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,16 +3128,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,12 +3148,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,12 +3273,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,12 +3348,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3362,7 +3362,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,12 +3498,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3553,16 +3553,16 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>116</v>
+        <v>67</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,12 +3623,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>106</v>
+        <v>77</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,23 +3698,123 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>85</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>16:34:35</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
+      <c r="C136" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D135" t="n">
-        <v>107</v>
-      </c>
-      <c r="E135" t="inlineStr">
+      <c r="D136" t="n">
+        <v>86</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>16:34:35</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>18:11</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>97</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>16:34:35</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>109</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>16:34:35</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>110</v>
+      </c>
+      <c r="E139" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3744,7 +3844,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:13:31</t>
+          <t>Última actualización: 16:34:35</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4335,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4249,7 +4349,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4285,7 +4385,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4299,7 +4399,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4310,7 +4410,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4324,7 +4424,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4343,7 +4443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4356,14 +4456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:13:31</t>
+          <t>Última actualización: 16:34:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4947,7 +5047,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4961,7 +5061,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4972,7 +5072,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4986,7 +5086,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5014,6 +5114,31 @@
         <v>43</v>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>16:34:35</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>111</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1344
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E139"/>
+  <dimension ref="A1:E147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:34:35</t>
+          <t>Última actualización: 16:47:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 134</t>
+          <t>Total filas: 142</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>80</v>
+        <v>16</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,12 +3373,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>38</v>
+        <v>80</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3453,16 +3453,16 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>116</v>
+        <v>50</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3703,16 +3703,16 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>86</v>
+        <v>116</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>97</v>
+        <v>61</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,23 +3798,223 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>64</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>72</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>73</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
           <t>16:34:35</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>18:11</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>97</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>85</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>96</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
         <is>
           <t>18:24</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
+      <c r="C145" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D139" t="n">
-        <v>110</v>
-      </c>
-      <c r="E139" t="inlineStr">
+      <c r="D145" t="n">
+        <v>97</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>108</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>112</v>
+      </c>
+      <c r="E147" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3831,7 +4031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3844,14 +4044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:34:35</t>
+          <t>Última actualización: 16:47:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4535,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4349,7 +4549,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4410,7 +4610,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4424,9 +4624,34 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>61</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4443,7 +4668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4456,14 +4681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:34:35</t>
+          <t>Última actualización: 16:47:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5322,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5111,7 +5336,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5139,6 +5364,31 @@
         <v>111</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>16:47:14</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>99</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1345
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E147"/>
+  <dimension ref="A1:E152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:14</t>
+          <t>Última actualización: 16:55:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 142</t>
+          <t>Total filas: 147</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3362,7 +3362,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>105</v>
+        <v>40</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,12 +3598,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>116</v>
+        <v>52</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>61</v>
+        <v>116</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,12 +3898,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3928,16 +3928,16 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,23 +3998,148 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
+          <t>16:55:33</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>100</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>16:55:33</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>18:38</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>103</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
           <t>16:47:14</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
+      <c r="B149" t="inlineStr">
         <is>
           <t>18:39</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
+      <c r="C149" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D147" t="n">
+      <c r="D149" t="n">
         <v>112</v>
       </c>
-      <c r="E147" t="inlineStr">
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>16:55:33</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>113</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>16:55:33</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>18:51</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>116</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>16:55:33</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>118</v>
+      </c>
+      <c r="E152" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4044,7 +4169,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:14</t>
+          <t>Última actualización: 16:55:33</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4660,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4549,7 +4674,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4585,7 +4710,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4599,7 +4724,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4620,7 +4745,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -4635,7 +4760,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4645,11 +4770,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4681,7 +4806,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:14</t>
+          <t>Última actualización: 16:55:33</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5447,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5336,7 +5461,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5372,7 +5497,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5386,7 +5511,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1346
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E152"/>
+  <dimension ref="A1:E157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:55:33</t>
+          <t>Última actualización: 17:13:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 147</t>
+          <t>Total filas: 152</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:13</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,12 +3473,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>46</v>
+        <v>84</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3903,16 +3903,16 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,12 +3923,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:13</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,23 +4123,148 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>95</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>17:13:28</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>18:51</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>98</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>17:13:28</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
           <t>18:53</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
+      <c r="C154" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D152" t="n">
-        <v>118</v>
-      </c>
-      <c r="E152" t="inlineStr">
+      <c r="D154" t="n">
+        <v>100</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>17:13:28</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>107</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>17:13:28</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>115</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>17:13:28</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>119</v>
+      </c>
+      <c r="E157" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4169,7 +4294,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:55:33</t>
+          <t>Última actualización: 17:13:28</t>
         </is>
       </c>
     </row>
@@ -4710,7 +4835,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4724,7 +4849,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4760,7 +4885,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4774,7 +4899,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4806,7 +4931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:55:33</t>
+          <t>Última actualización: 17:13:28</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5622,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5511,7 +5636,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1347
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E157"/>
+  <dimension ref="A1:E166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:13:28</t>
+          <t>Última actualización: 17:41:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 152</t>
+          <t>Total filas: 161</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,7 +3848,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,12 +3948,12 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>18:13</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4028,16 +4028,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:13</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>98</v>
+        <v>57</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>107</v>
+        <v>60</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4228,16 +4228,16 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,23 +4248,248 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
+          <t>18:51</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>70</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>72</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>18:58</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>77</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>79</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>87</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
           <t>19:12</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C162" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D157" t="n">
-        <v>119</v>
-      </c>
-      <c r="E157" t="inlineStr">
+      <c r="D162" t="n">
+        <v>91</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>96</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>102</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>103</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>115</v>
+      </c>
+      <c r="E166" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4281,7 +4506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4294,14 +4519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:13:28</t>
+          <t>Última actualización: 17:41:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4860,7 +5085,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4870,11 +5095,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4885,7 +5110,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4895,13 +5120,63 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>7</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>103</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>35</v>
-      </c>
-      <c r="E28" t="inlineStr">
+      <c r="D30" t="n">
+        <v>115</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4918,7 +5193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4931,14 +5206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:13:28</t>
+          <t>Última actualización: 17:41:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5641,6 +5916,56 @@
       <c r="E32" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>18:27</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>46</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>17:41:19</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>97</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1348
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E166"/>
+  <dimension ref="A1:E174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:41:19</t>
+          <t>Última actualización: 17:57:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 161</t>
+          <t>Total filas: 169</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3873,12 +3873,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3903,16 +3903,16 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>18:01</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3953,16 +3953,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,12 +3973,12 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>18:13</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:13</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,12 +4123,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:33</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>112</v>
+        <v>55</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>18:58</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,16 +4353,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:58</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>96</v>
+        <v>64</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>102</v>
+        <v>71</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,23 +4473,223 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>75</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>80</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>86</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>87</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
           <t>19:36</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C170" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D166" t="n">
-        <v>115</v>
-      </c>
-      <c r="E166" t="inlineStr">
+      <c r="D170" t="n">
+        <v>99</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>103</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>110</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>116</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>117</v>
+      </c>
+      <c r="E174" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4519,7 +4719,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:41:19</t>
+          <t>Última actualización: 17:57:34</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5335,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5149,7 +5349,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5160,7 +5360,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5174,7 +5374,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5193,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5206,14 +5406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:41:19</t>
+          <t>Última actualización: 17:57:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5947,23 +6147,48 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>34</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>19:18</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>97</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D35" t="n">
+        <v>81</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1349
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E174"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:57:34</t>
+          <t>Última actualización: 18:16:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 169</t>
+          <t>Total filas: 175</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>18:33</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:33</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,12 +4223,12 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>112</v>
+        <v>22</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>44</v>
+        <v>112</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>17:41:19</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>18:58</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>17:41:19</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:58</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4478,16 +4478,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>86</v>
+        <v>56</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4628,16 +4628,16 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4678,18 +4678,168 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>99</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>84</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>91</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>97</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
           <t>19:54</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
+      <c r="C178" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D174" t="n">
-        <v>117</v>
-      </c>
-      <c r="E174" t="inlineStr">
+      <c r="D178" t="n">
+        <v>98</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>104</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>118</v>
+      </c>
+      <c r="E180" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4706,7 +4856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4719,14 +4869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:57:34</t>
+          <t>Última actualización: 18:16:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5335,12 +5485,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5349,7 +5499,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5365,18 +5515,93 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>87</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>79</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>17:57:34</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>19:36</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D32" t="n">
         <v>99</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>118</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5393,7 +5618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5406,14 +5631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:57:34</t>
+          <t>Última actualización: 18:16:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -6147,12 +6372,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:29</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -6161,7 +6386,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6177,18 +6402,43 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>34</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>18:16:37</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>19:18</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>81</v>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D36" t="n">
+        <v>62</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1350
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:16:37</t>
+          <t>Última actualización: 18:35:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 175</t>
+          <t>Total filas: 180</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4312,7 +4312,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:03</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,12 +4498,12 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4528,16 +4528,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4603,16 +4603,16 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>87</v>
+        <v>48</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>79</v>
+        <v>48</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4678,16 +4678,16 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,16 +4703,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,23 +4823,148 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>78</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>18:35:37</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>79</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>18:35:37</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>85</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>18:35:37</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>96</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>18:35:37</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
           <t>20:14</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr">
+      <c r="C184" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D180" t="n">
-        <v>118</v>
-      </c>
-      <c r="E180" t="inlineStr">
+      <c r="D184" t="n">
+        <v>99</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>18:35:37</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>111</v>
+      </c>
+      <c r="E185" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4869,7 +4994,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:16:37</t>
+          <t>Última actualización: 18:35:37</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5610,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5499,7 +5624,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5560,7 +5685,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5574,7 +5699,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>99</v>
+        <v>61</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5585,7 +5710,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5599,7 +5724,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5631,7 +5756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:16:37</t>
+          <t>Última actualización: 18:35:37</t>
         </is>
       </c>
     </row>
@@ -6422,7 +6547,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6436,7 +6561,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1351
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E185"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:37</t>
+          <t>Última actualización: 18:48:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 180</t>
+          <t>Total filas: 189</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4312,7 +4312,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:06</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4628,16 +4628,16 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>79</v>
+        <v>48</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>99</v>
+        <v>65</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4953,18 +4953,243 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>79</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>67</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>72</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>83</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>18:35:37</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>99</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>87</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>18:35:37</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
           <t>20:26</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
+      <c r="C191" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D185" t="n">
+      <c r="D191" t="n">
         <v>111</v>
       </c>
-      <c r="E185" t="inlineStr">
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>99</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>107</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>116</v>
+      </c>
+      <c r="E194" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4981,7 +5206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4994,14 +5219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:37</t>
+          <t>Última actualización: 18:48:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5635,7 +5860,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5649,7 +5874,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5685,7 +5910,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5699,7 +5924,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5727,6 +5952,56 @@
         <v>99</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>87</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>116</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5743,7 +6018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5756,14 +6031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:37</t>
+          <t>Última actualización: 18:48:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6547,7 +6822,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6561,11 +6836,36 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>18:48:04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>117</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1352
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:04</t>
+          <t>Última actualización: 18:56:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 189</t>
+          <t>Total filas: 191</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,12 +4973,12 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>83</v>
+        <v>59</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5103,16 +5103,16 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,23 +5173,73 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>91</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>18:56:20</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>99</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>18:56:20</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
           <t>20:44</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
+      <c r="C196" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D194" t="n">
-        <v>116</v>
-      </c>
-      <c r="E194" t="inlineStr">
+      <c r="D196" t="n">
+        <v>108</v>
+      </c>
+      <c r="E196" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5219,7 +5269,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:04</t>
+          <t>Última actualización: 18:56:20</t>
         </is>
       </c>
     </row>
@@ -5860,7 +5910,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5874,7 +5924,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5910,7 +5960,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5924,7 +5974,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5960,7 +6010,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5974,7 +6024,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5985,7 +6035,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5999,7 +6049,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6031,7 +6081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:48:04</t>
+          <t>Última actualización: 18:56:20</t>
         </is>
       </c>
     </row>
@@ -6822,7 +6872,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6836,7 +6886,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6847,7 +6897,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6861,7 +6911,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1353
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E196"/>
+  <dimension ref="A1:E203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:56:20</t>
+          <t>Última actualización: 19:14:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 191</t>
+          <t>Total filas: 198</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,12 +4748,12 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>18:16:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>18:16:37</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,12 +4873,12 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5003,16 +5003,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>99</v>
+        <v>41</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5128,16 +5128,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>111</v>
+        <v>46</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,17 +5198,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5223,23 +5223,198 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>61</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>72</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
           <t>18:56:20</t>
         </is>
       </c>
-      <c r="B196" t="inlineStr">
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>91</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>81</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
         <is>
           <t>20:44</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr">
+      <c r="C200" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D196" t="n">
-        <v>108</v>
-      </c>
-      <c r="E196" t="inlineStr">
+      <c r="D200" t="n">
+        <v>90</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>101</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>101</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>21:11</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>117</v>
+      </c>
+      <c r="E203" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5256,7 +5431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5269,14 +5444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:56:20</t>
+          <t>Última actualización: 19:14:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -5910,7 +6085,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5924,7 +6099,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5960,7 +6135,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5974,7 +6149,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6010,7 +6185,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6024,7 +6199,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6035,7 +6210,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6049,9 +6224,34 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>101</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6068,7 +6268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6081,14 +6281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:56:20</t>
+          <t>Última actualización: 19:14:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6872,12 +7072,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6886,7 +7086,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6902,18 +7102,43 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>22</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>109</v>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="D38" t="n">
+        <v>91</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1354
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E203"/>
+  <dimension ref="A1:E215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:32</t>
+          <t>Última actualización: 19:41:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 198</t>
+          <t>Total filas: 210</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,12 +4998,12 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>18:48:04</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5078,16 +5078,16 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,12 +5098,12 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>18:48:04</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,12 +5123,12 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>99</v>
+        <v>19</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:04</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:09</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5303,16 +5303,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5353,16 +5353,16 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>101</v>
+        <v>45</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,23 +5398,323 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
+          <t>18:56:20</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>91</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>20:31</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>50</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>20:34</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>53</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
           <t>19:14:32</t>
         </is>
       </c>
-      <c r="B203" t="inlineStr">
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>81</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>63</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>74</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>101</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>75</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>20:59</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>78</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>79</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>19:14:32</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
         <is>
           <t>21:11</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr">
+      <c r="C213" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D203" t="n">
+      <c r="D213" t="n">
         <v>117</v>
       </c>
-      <c r="E203" t="inlineStr">
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>102</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>103</v>
+      </c>
+      <c r="E215" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5444,7 +5744,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:32</t>
+          <t>Última actualización: 19:41:55</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6460,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6174,7 +6474,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>99</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6210,7 +6510,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6224,7 +6524,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>90</v>
+        <v>63</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6235,7 +6535,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6249,7 +6549,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6268,7 +6568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6281,14 +6581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:32</t>
+          <t>Última actualización: 19:41:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7122,23 +7422,73 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>63</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>19:14:32</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>91</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>19:41:55</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>115</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1355
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E215"/>
+  <dimension ref="A1:E220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:41:55</t>
+          <t>Última actualización: 19:57:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 210</t>
+          <t>Total filas: 215</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4758,11 +4758,11 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>20:34</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,12 +5473,12 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,12 +5623,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>21:11</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>117</v>
+        <v>62</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5678,16 +5678,16 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>21:23</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,23 +5698,148 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
+          <t>21:11</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>117</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>21:13</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>76</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>86</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
           <t>21:24</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr">
+      <c r="C218" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D215" t="n">
-        <v>103</v>
-      </c>
-      <c r="E215" t="inlineStr">
+      <c r="D218" t="n">
+        <v>87</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>112</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>112</v>
+      </c>
+      <c r="E220" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5744,7 +5869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:41:55</t>
+          <t>Última actualización: 19:57:51</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6585,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6474,7 +6599,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6510,7 +6635,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6524,7 +6649,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6535,7 +6660,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6549,7 +6674,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6581,7 +6706,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:41:55</t>
+          <t>Última actualización: 19:57:51</t>
         </is>
       </c>
     </row>
@@ -7422,7 +7547,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7436,7 +7561,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7472,7 +7597,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7486,7 +7611,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1356
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E220"/>
+  <dimension ref="A1:E228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:51</t>
+          <t>Última actualización: 20:18:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 215</t>
+          <t>Total filas: 223</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:17:49</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>13:17:49</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>18:56:20</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:56:20</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,12 +5548,12 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>101</v>
+        <v>32</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>59</v>
+        <v>101</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,12 +5698,12 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>21:11</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -5712,7 +5712,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>117</v>
+        <v>39</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5728,16 +5728,16 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>21:13</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,16 +5753,16 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>21:23</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:11</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5828,18 +5828,218 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
+          <t>21:13</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>76</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>86</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>87</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>66</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>67</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>76</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
           <t>21:49</t>
         </is>
       </c>
-      <c r="C220" t="inlineStr">
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>91</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D220" t="n">
+      <c r="D227" t="n">
         <v>112</v>
       </c>
-      <c r="E220" t="inlineStr">
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>92</v>
+      </c>
+      <c r="E228" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5856,7 +6056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5869,14 +6069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:51</t>
+          <t>Última actualización: 20:18:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6585,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6395,11 +6595,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -6410,7 +6610,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -6420,11 +6620,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -6635,7 +6835,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6649,7 +6849,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6677,6 +6877,31 @@
         <v>58</v>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>38</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6693,7 +6918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6706,14 +6931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:57:51</t>
+          <t>Última actualización: 20:18:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7597,25 +7822,100 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>32</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>19:57:51</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>21:36</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D41" t="n">
         <v>99</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>79</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20:18:24</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>114</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1357
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E228"/>
+  <dimension ref="A1:E233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:24</t>
+          <t>Última actualización: 20:39:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 223</t>
+          <t>Total filas: 228</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>14:20:09</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>14:20:09</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:34:35</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>16:34:35</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5523,12 +5523,12 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5553,16 +5553,16 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>38</v>
+        <v>101</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,16 +5753,16 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>21:11</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>21:13</t>
+          <t>21:11</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5853,16 +5853,16 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>21:23</t>
+          <t>21:13</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>21:23</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>112</v>
+        <v>46</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,18 +6028,143 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>76</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>70</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>19:57:51</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>112</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
           <t>21:50</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr">
+      <c r="C231" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D228" t="n">
-        <v>92</v>
-      </c>
-      <c r="E228" t="inlineStr">
+      <c r="D231" t="n">
+        <v>71</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>100</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>108</v>
+      </c>
+      <c r="E233" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6056,7 +6181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6069,14 +6194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:24</t>
+          <t>Última actualización: 20:39:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6710,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6595,11 +6720,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -6610,7 +6735,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -6620,11 +6745,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -6835,12 +6960,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6849,7 +6974,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6860,21 +6985,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6885,23 +7010,73 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>58</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>38</v>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="D38" t="n">
+        <v>17</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>108</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6918,7 +7093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6931,14 +7106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:24</t>
+          <t>Última actualización: 20:39:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -7847,12 +8022,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -7861,7 +8036,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>99</v>
+        <v>15</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7872,12 +8047,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -7886,7 +8061,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7897,23 +8072,73 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>58</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>22:12</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>114</v>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="n">
+        <v>93</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20:39:01</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>113</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1358
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E233"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:39:01</t>
+          <t>Última actualización: 20:52:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 228</t>
+          <t>Total filas: 231</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>13:45:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:45:23</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>18:35:37</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>18:35:37</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4758,11 +4758,11 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5648,12 +5648,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -5662,7 +5662,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>5</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>21:11</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>21:13</t>
+          <t>21:11</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>21:22</t>
+          <t>21:13</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>21:23</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>86</v>
+        <v>43</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,12 +5948,12 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:23</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>87</v>
+        <v>32</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,12 +5998,12 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -6012,7 +6012,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>20:18:24</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:18:24</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:42</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>112</v>
+        <v>50</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>21:50</t>
+          <t>21:49</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>22:19</t>
+          <t>21:49</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,23 +6148,98 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
+          <t>20:52:18</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>58</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>20:52:18</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>87</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>20:52:18</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>94</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
           <t>20:39:01</t>
         </is>
       </c>
-      <c r="B233" t="inlineStr">
+      <c r="B236" t="inlineStr">
         <is>
           <t>22:27</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr">
+      <c r="C236" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D233" t="n">
+      <c r="D236" t="n">
         <v>108</v>
       </c>
-      <c r="E233" t="inlineStr">
+      <c r="E236" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6181,7 +6256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6194,14 +6269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:39:01</t>
+          <t>Última actualización: 20:52:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7110,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7049,7 +7124,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7060,23 +7135,48 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>20:52:18</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>94</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>20:39:01</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>22:27</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D40" t="n">
         <v>108</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7106,7 +7206,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:39:01</t>
+          <t>Última actualización: 20:52:18</t>
         </is>
       </c>
     </row>
@@ -8022,7 +8122,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8036,7 +8136,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8072,7 +8172,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8086,7 +8186,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8097,7 +8197,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8111,7 +8211,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8122,7 +8222,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8136,7 +8236,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1359
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-07.xlsx
+++ b/data/horarios-141-2026-03-07.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:52:18</t>
+          <t>Última actualización: 22:05:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 231</t>
+          <t>Total filas: 240</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12:56:14</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>12:56:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>14:55:32</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>14:55:32</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>13:58:57</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2</v>
+        <v>115</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>13:58:57</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>115</v>
+        <v>2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>16:55:33</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>16:55:33</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>16:13:31</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:13:31</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>17:57:34</t>
+          <t>16:47:14</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>16:47:14</t>
+          <t>17:57:34</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:41:55</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>19:41:55</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>19:14:32</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>19:14:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>20:52:18</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>20:52:18</t>
+          <t>20:39:01</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>20:39:01</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>20:52:18</t>
+          <t>19:57:51</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>32</v>
+        <v>87</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>19:57:51</t>
+          <t>20:52:18</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>87</v>
+        <v>32</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>20:52:18</t>
+          <t>22:05:16</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>22:19</t>
+          <t>22:17</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>87</v>
+        <v>12</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>20:52:18</t>
+          <t>22:05:16</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>22:26</t>
+          <t>22:19</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,23 +6223,248 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>22:20</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>15</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>21</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
           <t>20:39:01</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
+      <c r="B238" t="inlineStr">
         <is>
           <t>22:27</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
+      <c r="C238" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D236" t="n">
+      <c r="D238" t="n">
         <v>108</v>
       </c>
-      <c r="E236" t="inlineStr">
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>32</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>22:49</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>44</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>22:59</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>54</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>23:10</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>65</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>23:19</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>74</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>23:44</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>99</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>23:49</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>104</v>
+      </c>
+      <c r="E245" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6256,7 +6481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6269,14 +6494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:52:18</t>
+          <t>Última actualización: 22:05:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -6785,7 +7010,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>15:51:56</t>
+          <t>17:13:28</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6795,11 +7020,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -6810,7 +7035,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>17:13:28</t>
+          <t>15:51:56</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -6820,11 +7045,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -7135,7 +7360,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>20:52:18</t>
+          <t>22:05:16</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7149,7 +7374,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>94</v>
+        <v>21</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7177,6 +7402,31 @@
         <v>108</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>22:05:16</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>23:44</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>99</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7206,7 +7456,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:52:18</t>
+          <t>Última actualización: 22:05:16</t>
         </is>
       </c>
     </row>
@@ -8197,7 +8447,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20:52:18</t>
+          <t>22:05:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8211,7 +8461,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>80</v>
+        <v>7</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8222,7 +8472,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20:52:18</t>
+          <t>22:05:16</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8236,7 +8486,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>

</xml_diff>